<commit_message>
2019년도 static featre 생성 완료
</commit_message>
<xml_diff>
--- a/dataset/raw/dong/mismatch_report_2019.xlsx
+++ b/dataset/raw/dong/mismatch_report_2019.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10719"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24F6162-A1DC-2548-B8C5-FBCE082D014F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CE80B1-5EEB-2C44-9CD5-1C656ADE22FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23600" yWindow="6640" windowWidth="23600" windowHeight="12940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1761" uniqueCount="1432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1765" uniqueCount="1434">
   <si>
     <t>동이름</t>
   </si>
@@ -3948,10 +3948,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>신31240700/신31240690/신31240710</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>신31130160</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -4276,14 +4272,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>감북동-&gt;감북동/감일동, 감일동-&gt;감일동/상일2동</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>신31180660/신31180670/신11250770</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>영종동-&gt;영종동/영종1동/영종2동</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -4564,10 +4552,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>신31240700/신31240690/신31240710/신31240720</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>상현1동-&gt;상현1동/상현3동</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -4633,6 +4617,30 @@
   </si>
   <si>
     <t>영통1동, 영통2동 -&gt; 영통1동/영통2동/영통3동</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>신11250750/신11250770</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>강일동-&gt;상일2동</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>신31180660/신31180670</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>감북동-&gt;감북동/감일동</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>신31240700/신31240690/신31240710/신31240691</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>신31240700/신31240690/신31240710/신31240720/신31240691</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -5100,7 +5108,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="24" width="13.5" customWidth="1"/>
+    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="24" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9787,16 +9797,16 @@
         <v>11170730</v>
       </c>
       <c r="C275" s="4" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D275" s="4" t="s">
+        <v>1264</v>
+      </c>
+      <c r="E275" s="4" t="s">
+        <v>1264</v>
+      </c>
+      <c r="F275" s="4" t="s">
         <v>1265</v>
-      </c>
-      <c r="D275" s="4" t="s">
-        <v>1265</v>
-      </c>
-      <c r="E275" s="4" t="s">
-        <v>1265</v>
-      </c>
-      <c r="F275" s="4" t="s">
-        <v>1266</v>
       </c>
     </row>
     <row r="276" spans="1:6">
@@ -11561,13 +11571,13 @@
         <v>11230740</v>
       </c>
       <c r="D379" s="4" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="E379">
         <v>11230740</v>
       </c>
       <c r="F379" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="380" spans="1:6">
@@ -12053,14 +12063,17 @@
       <c r="B408">
         <v>11250750</v>
       </c>
-      <c r="C408">
-        <v>11250750</v>
-      </c>
-      <c r="D408">
-        <v>11250750</v>
-      </c>
-      <c r="E408">
-        <v>11250750</v>
+      <c r="C408" s="4" t="s">
+        <v>1428</v>
+      </c>
+      <c r="D408" s="4" t="s">
+        <v>1428</v>
+      </c>
+      <c r="E408" s="4" t="s">
+        <v>1428</v>
+      </c>
+      <c r="F408" t="s">
+        <v>1429</v>
       </c>
     </row>
     <row r="409" spans="1:6">
@@ -12071,16 +12084,16 @@
         <v>1174052000</v>
       </c>
       <c r="C409" s="4" t="s">
+        <v>1339</v>
+      </c>
+      <c r="D409" s="4" t="s">
+        <v>1339</v>
+      </c>
+      <c r="E409" s="4" t="s">
+        <v>1339</v>
+      </c>
+      <c r="F409" s="4" t="s">
         <v>1340</v>
-      </c>
-      <c r="D409" s="4" t="s">
-        <v>1340</v>
-      </c>
-      <c r="E409" s="4" t="s">
-        <v>1340</v>
-      </c>
-      <c r="F409" s="4" t="s">
-        <v>1341</v>
       </c>
     </row>
     <row r="410" spans="1:6">
@@ -12465,16 +12478,16 @@
         <v>2811060000</v>
       </c>
       <c r="C432" s="4" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="D432" s="4" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="E432" s="4" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="F432" t="s">
-        <v>1347</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="433" spans="1:6">
@@ -12485,16 +12498,16 @@
         <v>2811061000</v>
       </c>
       <c r="C433" s="4" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="D433" s="4" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="E433" s="4" t="s">
-        <v>1349</v>
+        <v>1346</v>
       </c>
       <c r="F433" t="s">
-        <v>1348</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="434" spans="1:6">
@@ -12505,16 +12518,16 @@
         <v>23010650</v>
       </c>
       <c r="C434" s="4" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="D434" s="4" t="s">
-        <v>1346</v>
+        <v>1343</v>
       </c>
       <c r="E434" s="4" t="s">
-        <v>1345</v>
+        <v>1342</v>
       </c>
       <c r="F434" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="435" spans="1:6">
@@ -13353,16 +13366,16 @@
         <v>23040660</v>
       </c>
       <c r="C480" s="4" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="D480" s="4" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="E480" s="4" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="F480" s="4" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="481" spans="1:6">
@@ -13410,7 +13423,7 @@
         <v>23050520</v>
       </c>
       <c r="D483" s="4" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="E483">
         <v>23050520</v>
@@ -13478,7 +13491,7 @@
         <v>23050560</v>
       </c>
       <c r="D487" s="4" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="E487">
         <v>23050560</v>
@@ -14314,7 +14327,7 @@
         <v>23080530</v>
       </c>
       <c r="D536" s="4" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="E536">
         <v>23080530</v>
@@ -14382,7 +14395,7 @@
         <v>23080540</v>
       </c>
       <c r="D540" s="4" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="E540">
         <v>23080540</v>
@@ -14609,16 +14622,16 @@
         <v>2826065000</v>
       </c>
       <c r="C553" s="3" t="s">
-        <v>1351</v>
+        <v>1348</v>
       </c>
       <c r="D553" s="3" t="s">
-        <v>1351</v>
+        <v>1348</v>
       </c>
       <c r="E553" s="3" t="s">
-        <v>1351</v>
+        <v>1348</v>
       </c>
       <c r="F553" s="3" t="s">
-        <v>1350</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -14629,16 +14642,16 @@
         <v>2826066000</v>
       </c>
       <c r="C554" s="4" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="D554" s="4" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="E554" s="4" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="F554" s="4" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="555" spans="1:12">
@@ -14669,13 +14682,13 @@
         <v>23510110</v>
       </c>
       <c r="C556" s="4" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="D556">
         <v>23510110</v>
       </c>
       <c r="E556" s="4" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="557" spans="1:12">
@@ -14686,13 +14699,13 @@
         <v>23510310</v>
       </c>
       <c r="C557" s="4" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="D557">
         <v>23510310</v>
       </c>
       <c r="E557" s="4" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="G557" s="2"/>
     </row>
@@ -14704,13 +14717,13 @@
         <v>23510320</v>
       </c>
       <c r="C558" s="4" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="D558">
         <v>23510320</v>
       </c>
       <c r="E558" s="4" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="559" spans="1:12">
@@ -14721,13 +14734,13 @@
         <v>23510330</v>
       </c>
       <c r="C559" s="4" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="D559">
         <v>23510330</v>
       </c>
       <c r="E559" s="4" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="560" spans="1:12">
@@ -14738,13 +14751,13 @@
         <v>23510340</v>
       </c>
       <c r="C560" s="4" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="D560">
         <v>23510340</v>
       </c>
       <c r="E560" s="4" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="561" spans="1:9">
@@ -14755,13 +14768,13 @@
         <v>23510350</v>
       </c>
       <c r="C561" s="4" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="D561">
         <v>23510350</v>
       </c>
       <c r="E561" s="4" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="562" spans="1:9">
@@ -14772,13 +14785,13 @@
         <v>23510360</v>
       </c>
       <c r="C562" s="4" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D562">
         <v>23510360</v>
       </c>
       <c r="E562" s="4" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="563" spans="1:9">
@@ -14789,13 +14802,13 @@
         <v>23510370</v>
       </c>
       <c r="C563" s="4" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="D563">
         <v>23510370</v>
       </c>
       <c r="E563" s="4" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="564" spans="1:9">
@@ -14806,13 +14819,13 @@
         <v>23510380</v>
       </c>
       <c r="C564" s="4" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="D564">
         <v>23510380</v>
       </c>
       <c r="E564" s="4" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="565" spans="1:9">
@@ -14823,13 +14836,13 @@
         <v>23510390</v>
       </c>
       <c r="C565" s="4" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="D565">
         <v>23510390</v>
       </c>
       <c r="E565" s="4" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="566" spans="1:9">
@@ -14840,13 +14853,13 @@
         <v>23510400</v>
       </c>
       <c r="C566" s="4" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="D566">
         <v>23510400</v>
       </c>
       <c r="E566" s="4" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="567" spans="1:9">
@@ -14857,13 +14870,13 @@
         <v>23510410</v>
       </c>
       <c r="C567" s="4" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="D567">
         <v>23510410</v>
       </c>
       <c r="E567" s="4" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="568" spans="1:9">
@@ -14874,13 +14887,13 @@
         <v>23510420</v>
       </c>
       <c r="C568" s="4" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="D568">
         <v>23510420</v>
       </c>
       <c r="E568" s="4" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="569" spans="1:9">
@@ -14891,13 +14904,13 @@
         <v>23520310</v>
       </c>
       <c r="C569" s="4" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="D569">
         <v>23520310</v>
       </c>
       <c r="E569" s="4" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="570" spans="1:9">
@@ -14908,13 +14921,13 @@
         <v>23520330</v>
       </c>
       <c r="C570" s="4" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="D570">
         <v>23520330</v>
       </c>
       <c r="E570" s="4" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="571" spans="1:9">
@@ -14925,13 +14938,13 @@
         <v>23520340</v>
       </c>
       <c r="C571" s="4" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="D571">
         <v>23520340</v>
       </c>
       <c r="E571" s="4" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="572" spans="1:9">
@@ -14942,13 +14955,13 @@
         <v>23520350</v>
       </c>
       <c r="C572" s="4" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="D572">
         <v>23520350</v>
       </c>
       <c r="E572" s="4" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="573" spans="1:9">
@@ -14959,13 +14972,13 @@
         <v>23520370</v>
       </c>
       <c r="C573" s="4" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="D573">
         <v>23520370</v>
       </c>
       <c r="E573" s="4" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="574" spans="1:9">
@@ -14976,13 +14989,13 @@
         <v>23520360</v>
       </c>
       <c r="C574" s="4" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="D574">
         <v>23520360</v>
       </c>
       <c r="E574" s="4" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="I574" s="9"/>
     </row>
@@ -14994,13 +15007,13 @@
         <v>23520320</v>
       </c>
       <c r="C575" s="4" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="D575">
         <v>23520320</v>
       </c>
       <c r="E575" s="4" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="576" spans="1:9">
@@ -15640,16 +15653,16 @@
         <v>31014640</v>
       </c>
       <c r="C613" s="4" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="D613" s="4" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="E613" s="4" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="F613" t="s">
-        <v>1431</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="614" spans="1:11">
@@ -15660,16 +15673,16 @@
         <v>31014650</v>
       </c>
       <c r="C614" s="4" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="D614" s="4" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="E614" s="4" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="F614" t="s">
-        <v>1431</v>
+        <v>1427</v>
       </c>
       <c r="G614" s="2"/>
       <c r="H614" s="2"/>
@@ -16626,16 +16639,16 @@
         <v>4115053000</v>
       </c>
       <c r="C670" s="4" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
       <c r="D670" s="4" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
       <c r="E670" s="4" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
       <c r="F670" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="671" spans="1:6">
@@ -16737,13 +16750,13 @@
         <v>31030590</v>
       </c>
       <c r="D676" s="4" t="s">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="E676">
         <v>31030590</v>
       </c>
       <c r="F676" t="s">
-        <v>1352</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="677" spans="1:10">
@@ -16754,16 +16767,16 @@
         <v>31030700</v>
       </c>
       <c r="C677" s="4" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="D677" s="4" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="E677" s="4" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="F677" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="678" spans="1:10">
@@ -17060,13 +17073,13 @@
         <v>31041620</v>
       </c>
       <c r="D694" s="4" t="s">
-        <v>1354</v>
+        <v>1351</v>
       </c>
       <c r="E694">
         <v>31041620</v>
       </c>
       <c r="F694" t="s">
-        <v>1355</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="695" spans="1:6">
@@ -17199,13 +17212,13 @@
         <v>31042560</v>
       </c>
       <c r="D702" s="4" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="E702">
         <v>31042560</v>
       </c>
       <c r="F702" t="s">
-        <v>1358</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="703" spans="1:6">
@@ -17219,13 +17232,13 @@
         <v>31042570</v>
       </c>
       <c r="D703" s="7" t="s">
-        <v>1356</v>
+        <v>1353</v>
       </c>
       <c r="E703">
         <v>31042570</v>
       </c>
       <c r="F703" t="s">
-        <v>1357</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="704" spans="1:6">
@@ -17946,13 +17959,13 @@
         <v>1211</v>
       </c>
       <c r="D741" s="4" t="s">
-        <v>1360</v>
+        <v>1357</v>
       </c>
       <c r="E741" s="4" t="s">
         <v>1211</v>
       </c>
       <c r="F741" t="s">
-        <v>1359</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="742" spans="1:10">
@@ -18404,16 +18417,16 @@
         <v>31060690</v>
       </c>
       <c r="C766" s="4" t="s">
-        <v>1361</v>
+        <v>1358</v>
       </c>
       <c r="D766" s="4" t="s">
-        <v>1361</v>
+        <v>1358</v>
       </c>
       <c r="E766" s="4" t="s">
-        <v>1361</v>
+        <v>1358</v>
       </c>
       <c r="F766" s="4" t="s">
-        <v>1362</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="767" spans="1:6">
@@ -18543,16 +18556,16 @@
         <v>31070330</v>
       </c>
       <c r="C774" s="4" t="s">
-        <v>1363</v>
+        <v>1360</v>
       </c>
       <c r="D774" s="4" t="s">
-        <v>1363</v>
+        <v>1360</v>
       </c>
       <c r="E774" s="4" t="s">
-        <v>1363</v>
+        <v>1360</v>
       </c>
       <c r="F774" s="4" t="s">
-        <v>1364</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="775" spans="1:6">
@@ -18767,16 +18780,16 @@
         <v>31070670</v>
       </c>
       <c r="C787" s="4" t="s">
-        <v>1370</v>
+        <v>1367</v>
       </c>
       <c r="D787" s="4" t="s">
-        <v>1370</v>
+        <v>1367</v>
       </c>
       <c r="E787" s="4" t="s">
-        <v>1370</v>
+        <v>1367</v>
       </c>
       <c r="F787" s="4" t="s">
-        <v>1371</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="788" spans="1:6">
@@ -18994,16 +19007,16 @@
         <v>4127152000</v>
       </c>
       <c r="C800" s="4" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="D800" s="4" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="E800" s="4" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="F800" s="4" t="s">
-        <v>1369</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="801" spans="1:6">
@@ -19014,16 +19027,16 @@
         <v>4127153000</v>
       </c>
       <c r="C801" s="4" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
       <c r="D801" s="4" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
       <c r="E801" s="4" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
       <c r="F801" s="4" t="s">
-        <v>1365</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="802" spans="1:6">
@@ -19034,16 +19047,16 @@
         <v>4127153500</v>
       </c>
       <c r="C802" s="3" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="D802" s="3" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="E802" s="3" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="F802" s="3" t="s">
-        <v>1368</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="803" spans="1:6">
@@ -19207,16 +19220,16 @@
         <v>4127352000</v>
       </c>
       <c r="C812" s="4" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="D812" s="4" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="E812" s="4" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="F812" s="4" t="s">
-        <v>1374</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="813" spans="1:6">
@@ -19227,16 +19240,16 @@
         <v>4127353000</v>
       </c>
       <c r="C813" s="3" t="s">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="D813" s="3" t="s">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="E813" s="3" t="s">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="F813" s="4" t="s">
-        <v>1372</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="814" spans="1:6">
@@ -19446,13 +19459,13 @@
         <v>31101530</v>
       </c>
       <c r="D825" s="4" t="s">
-        <v>1421</v>
+        <v>1417</v>
       </c>
       <c r="E825">
         <v>31101530</v>
       </c>
       <c r="F825" t="s">
-        <v>1423</v>
+        <v>1419</v>
       </c>
       <c r="H825" s="2"/>
     </row>
@@ -19519,13 +19532,13 @@
         <v>31101700</v>
       </c>
       <c r="D829" s="4" t="s">
-        <v>1422</v>
+        <v>1418</v>
       </c>
       <c r="E829">
         <v>31101700</v>
       </c>
       <c r="F829" t="s">
-        <v>1424</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="830" spans="1:8">
@@ -19692,13 +19705,13 @@
         <v>31101690</v>
       </c>
       <c r="D839" s="4" t="s">
-        <v>1376</v>
+        <v>1373</v>
       </c>
       <c r="E839">
         <v>31101690</v>
       </c>
       <c r="F839" t="s">
-        <v>1375</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="840" spans="1:8">
@@ -19763,13 +19776,13 @@
         <v>31103520</v>
       </c>
       <c r="D843" s="4" t="s">
-        <v>1378</v>
+        <v>1375</v>
       </c>
       <c r="E843">
         <v>31103520</v>
       </c>
       <c r="F843" t="s">
-        <v>1377</v>
+        <v>1374</v>
       </c>
       <c r="H843" s="2"/>
     </row>
@@ -19989,13 +20002,13 @@
         <v>31104540</v>
       </c>
       <c r="D856" s="4" t="s">
-        <v>1379</v>
+        <v>1376</v>
       </c>
       <c r="E856">
         <v>31104540</v>
       </c>
       <c r="F856" t="s">
-        <v>1380</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="857" spans="1:8">
@@ -20077,13 +20090,13 @@
         <v>31104590</v>
       </c>
       <c r="D861" s="4" t="s">
-        <v>1382</v>
+        <v>1379</v>
       </c>
       <c r="E861">
         <v>31104590</v>
       </c>
       <c r="F861" t="s">
-        <v>1381</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="862" spans="1:8">
@@ -20114,13 +20127,13 @@
         <v>31110520</v>
       </c>
       <c r="D863" s="4" t="s">
-        <v>1384</v>
+        <v>1381</v>
       </c>
       <c r="E863">
         <v>31110520</v>
       </c>
       <c r="F863" t="s">
-        <v>1383</v>
+        <v>1380</v>
       </c>
       <c r="H863" s="2"/>
     </row>
@@ -20473,16 +20486,16 @@
         <v>4136037000</v>
       </c>
       <c r="C884" s="4" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D884" s="4" t="s">
+        <v>1260</v>
+      </c>
+      <c r="E884" s="4" t="s">
+        <v>1260</v>
+      </c>
+      <c r="F884" s="4" t="s">
         <v>1261</v>
-      </c>
-      <c r="D884" s="4" t="s">
-        <v>1261</v>
-      </c>
-      <c r="E884" s="4" t="s">
-        <v>1261</v>
-      </c>
-      <c r="F884" s="4" t="s">
-        <v>1262</v>
       </c>
     </row>
     <row r="885" spans="1:7">
@@ -20564,13 +20577,13 @@
         <v>31130590</v>
       </c>
       <c r="D889" s="4" t="s">
-        <v>1387</v>
+        <v>1384</v>
       </c>
       <c r="E889">
         <v>31130590</v>
       </c>
       <c r="F889" t="s">
-        <v>1386</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="890" spans="1:7">
@@ -20584,13 +20597,13 @@
         <v>31130580</v>
       </c>
       <c r="D890" s="4" t="s">
-        <v>1388</v>
+        <v>1385</v>
       </c>
       <c r="E890">
         <v>31130580</v>
       </c>
       <c r="F890" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="891" spans="1:7">
@@ -20655,13 +20668,13 @@
         <v>31140540</v>
       </c>
       <c r="D894" s="4" t="s">
-        <v>1390</v>
+        <v>1387</v>
       </c>
       <c r="E894">
         <v>31140540</v>
       </c>
       <c r="F894" t="s">
-        <v>1389</v>
+        <v>1386</v>
       </c>
       <c r="G894" s="8"/>
     </row>
@@ -20710,13 +20723,13 @@
         <v>31140520</v>
       </c>
       <c r="D897" s="4" t="s">
-        <v>1392</v>
+        <v>1389</v>
       </c>
       <c r="E897">
         <v>31140520</v>
       </c>
       <c r="F897" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="898" spans="1:7">
@@ -20868,13 +20881,13 @@
         <v>31150640</v>
       </c>
       <c r="D906" s="4" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
       <c r="E906">
         <v>31150640</v>
       </c>
       <c r="F906" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="907" spans="1:7">
@@ -20936,16 +20949,16 @@
         <v>31150720</v>
       </c>
       <c r="C910" s="4" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="D910" s="4" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="E910" s="4" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="F910" t="s">
-        <v>1396</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="911" spans="1:7">
@@ -21041,16 +21054,16 @@
         <v>31160520</v>
       </c>
       <c r="C916" s="4" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="D916" s="4" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="E916" s="4" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="F916" t="s">
-        <v>1417</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="917" spans="1:6">
@@ -21421,7 +21434,7 @@
         <v>31180610</v>
       </c>
       <c r="D938" s="4" t="s">
-        <v>1425</v>
+        <v>1421</v>
       </c>
       <c r="E938">
         <v>31180610</v>
@@ -21435,16 +21448,16 @@
         <v>31180660</v>
       </c>
       <c r="C939" s="4" t="s">
-        <v>1343</v>
+        <v>1430</v>
       </c>
       <c r="D939" s="4" t="s">
-        <v>1343</v>
+        <v>1430</v>
       </c>
       <c r="E939" s="4" t="s">
-        <v>1343</v>
+        <v>1430</v>
       </c>
       <c r="F939" s="4" t="s">
-        <v>1342</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="940" spans="1:6">
@@ -21577,16 +21590,16 @@
         <v>4146132000</v>
       </c>
       <c r="C947" s="4" t="s">
-        <v>1398</v>
+        <v>1395</v>
       </c>
       <c r="D947" s="4" t="s">
-        <v>1398</v>
+        <v>1395</v>
       </c>
       <c r="E947" s="4" t="s">
-        <v>1398</v>
+        <v>1395</v>
       </c>
       <c r="F947" t="s">
-        <v>1397</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="948" spans="1:10">
@@ -21685,16 +21698,16 @@
         <v>4146152000</v>
       </c>
       <c r="C953" s="4" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
       <c r="D953" s="4" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
       <c r="E953" s="4" t="s">
-        <v>1400</v>
+        <v>1397</v>
       </c>
       <c r="F953" t="s">
-        <v>1399</v>
+        <v>1396</v>
       </c>
       <c r="H953" s="2"/>
       <c r="I953" s="2"/>
@@ -21759,16 +21772,16 @@
         <v>4146351500</v>
       </c>
       <c r="C957" s="4" t="s">
+        <v>1268</v>
+      </c>
+      <c r="D957" s="4" t="s">
+        <v>1268</v>
+      </c>
+      <c r="E957" s="4" t="s">
+        <v>1268</v>
+      </c>
+      <c r="F957" s="4" t="s">
         <v>1269</v>
-      </c>
-      <c r="D957" s="4" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E957" s="4" t="s">
-        <v>1269</v>
-      </c>
-      <c r="F957" s="4" t="s">
-        <v>1270</v>
       </c>
     </row>
     <row r="958" spans="1:10">
@@ -21796,16 +21809,16 @@
         <v>31192650</v>
       </c>
       <c r="C959" s="4" t="s">
+        <v>1270</v>
+      </c>
+      <c r="D959" s="4" t="s">
+        <v>1270</v>
+      </c>
+      <c r="E959" s="4" t="s">
+        <v>1270</v>
+      </c>
+      <c r="F959" s="4" t="s">
         <v>1271</v>
-      </c>
-      <c r="D959" s="4" t="s">
-        <v>1271</v>
-      </c>
-      <c r="E959" s="4" t="s">
-        <v>1271</v>
-      </c>
-      <c r="F959" s="4" t="s">
-        <v>1272</v>
       </c>
     </row>
     <row r="960" spans="1:10">
@@ -21884,16 +21897,16 @@
         <v>4146358500</v>
       </c>
       <c r="C964" s="4" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D964" s="4" t="s">
+        <v>1272</v>
+      </c>
+      <c r="E964" s="4" t="s">
+        <v>1272</v>
+      </c>
+      <c r="F964" s="4" t="s">
         <v>1273</v>
-      </c>
-      <c r="D964" s="4" t="s">
-        <v>1273</v>
-      </c>
-      <c r="E964" s="4" t="s">
-        <v>1273</v>
-      </c>
-      <c r="F964" s="4" t="s">
-        <v>1274</v>
       </c>
     </row>
     <row r="965" spans="1:6">
@@ -21989,16 +22002,16 @@
         <v>31193600</v>
       </c>
       <c r="C970" s="4" t="s">
-        <v>1402</v>
+        <v>1399</v>
       </c>
       <c r="D970" s="4" t="s">
-        <v>1402</v>
+        <v>1399</v>
       </c>
       <c r="E970" s="4" t="s">
-        <v>1402</v>
+        <v>1399</v>
       </c>
       <c r="F970" t="s">
-        <v>1401</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="971" spans="1:6">
@@ -22043,16 +22056,16 @@
         <v>31193620</v>
       </c>
       <c r="C973" s="4" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
       <c r="D973" s="4" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
       <c r="E973" s="4" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
       <c r="F973" t="s">
-        <v>1415</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="974" spans="1:6">
@@ -22250,16 +22263,16 @@
         <v>4148038000</v>
       </c>
       <c r="C985" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="D985" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="E985" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="F985" s="4" t="s">
-        <v>1429</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="986" spans="1:6">
@@ -22287,16 +22300,16 @@
         <v>4148040000</v>
       </c>
       <c r="C987" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="D987" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="E987" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="F987" s="4" t="s">
-        <v>1428</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="988" spans="1:6">
@@ -22307,16 +22320,16 @@
         <v>4148041000</v>
       </c>
       <c r="C988" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="D988" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="E988" s="4" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="F988" s="4" t="s">
-        <v>1427</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="989" spans="1:6">
@@ -22381,13 +22394,13 @@
         <v>31200550</v>
       </c>
       <c r="D992" s="4" t="s">
-        <v>1411</v>
+        <v>1408</v>
       </c>
       <c r="E992">
         <v>31200550</v>
       </c>
       <c r="F992" t="s">
-        <v>1412</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="993" spans="1:6">
@@ -22435,13 +22448,13 @@
         <v>31200580</v>
       </c>
       <c r="D995" s="4" t="s">
-        <v>1409</v>
+        <v>1406</v>
       </c>
       <c r="E995">
         <v>31200580</v>
       </c>
       <c r="F995" t="s">
-        <v>1410</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="996" spans="1:6">
@@ -23403,16 +23416,16 @@
         <v>4159042000</v>
       </c>
       <c r="C1051" s="4" t="s">
-        <v>1260</v>
+        <v>1432</v>
       </c>
       <c r="D1051" s="4" t="s">
-        <v>1414</v>
+        <v>1433</v>
       </c>
       <c r="E1051" s="4" t="s">
-        <v>1260</v>
+        <v>1432</v>
       </c>
       <c r="F1051" s="4" t="s">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="1052" spans="1:10">
@@ -23599,13 +23612,13 @@
         <v>31250110</v>
       </c>
       <c r="D1062" s="4" t="s">
-        <v>1408</v>
+        <v>1405</v>
       </c>
       <c r="E1062">
         <v>31250110</v>
       </c>
       <c r="F1062" t="s">
-        <v>1407</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="1063" spans="1:13">
@@ -23734,16 +23747,16 @@
         <v>31250540</v>
       </c>
       <c r="C1069" s="4" t="s">
+        <v>1276</v>
+      </c>
+      <c r="D1069" s="4" t="s">
+        <v>1276</v>
+      </c>
+      <c r="E1069" s="4" t="s">
+        <v>1276</v>
+      </c>
+      <c r="F1069" s="4" t="s">
         <v>1277</v>
-      </c>
-      <c r="D1069" s="4" t="s">
-        <v>1277</v>
-      </c>
-      <c r="E1069" s="4" t="s">
-        <v>1277</v>
-      </c>
-      <c r="F1069" s="4" t="s">
-        <v>1278</v>
       </c>
     </row>
     <row r="1070" spans="1:13">
@@ -23754,16 +23767,16 @@
         <v>31250550</v>
       </c>
       <c r="C1070" s="4" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D1070" s="4" t="s">
+        <v>1278</v>
+      </c>
+      <c r="E1070" s="4" t="s">
+        <v>1278</v>
+      </c>
+      <c r="F1070" s="4" t="s">
         <v>1279</v>
-      </c>
-      <c r="D1070" s="4" t="s">
-        <v>1279</v>
-      </c>
-      <c r="E1070" s="4" t="s">
-        <v>1279</v>
-      </c>
-      <c r="F1070" s="4" t="s">
-        <v>1280</v>
       </c>
     </row>
     <row r="1071" spans="1:13">
@@ -23774,16 +23787,16 @@
         <v>4161053000</v>
       </c>
       <c r="C1071" s="4" t="s">
+        <v>1280</v>
+      </c>
+      <c r="D1071" s="4" t="s">
+        <v>1280</v>
+      </c>
+      <c r="E1071" s="4" t="s">
+        <v>1280</v>
+      </c>
+      <c r="F1071" s="4" t="s">
         <v>1281</v>
-      </c>
-      <c r="D1071" s="4" t="s">
-        <v>1281</v>
-      </c>
-      <c r="E1071" s="4" t="s">
-        <v>1281</v>
-      </c>
-      <c r="F1071" s="4" t="s">
-        <v>1282</v>
       </c>
     </row>
     <row r="1072" spans="1:13">
@@ -23967,13 +23980,13 @@
         <v>31260560</v>
       </c>
       <c r="D1082" s="10" t="s">
-        <v>1406</v>
+        <v>1403</v>
       </c>
       <c r="E1082">
         <v>31260560</v>
       </c>
       <c r="F1082" t="s">
-        <v>1405</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="1083" spans="1:6">
@@ -24290,16 +24303,16 @@
         <v>4167034000</v>
       </c>
       <c r="C1101" s="4" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="D1101" s="4" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="E1101" s="4" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="F1101" s="4" t="s">
-        <v>1404</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="1102" spans="1:6">
@@ -24429,13 +24442,13 @@
         <v>31550110</v>
       </c>
       <c r="C1109" s="4" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="D1109">
         <v>31550110</v>
       </c>
       <c r="E1109" s="4" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="1110" spans="1:5">
@@ -24446,13 +24459,13 @@
         <v>31550120</v>
       </c>
       <c r="C1110" s="4" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="D1110">
         <v>31550120</v>
       </c>
       <c r="E1110" s="4" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="1111" spans="1:5">
@@ -24463,13 +24476,13 @@
         <v>31550310</v>
       </c>
       <c r="C1111" s="4" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="D1111">
         <v>31550310</v>
       </c>
       <c r="E1111" s="4" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="1112" spans="1:5">
@@ -24480,13 +24493,13 @@
         <v>31550320</v>
       </c>
       <c r="C1112" s="4" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="D1112">
         <v>31550320</v>
       </c>
       <c r="E1112" s="4" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="1113" spans="1:5">
@@ -24497,13 +24510,13 @@
         <v>31550330</v>
       </c>
       <c r="C1113" s="4" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="D1113">
         <v>31550330</v>
       </c>
       <c r="E1113" s="4" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="1114" spans="1:5">
@@ -24514,13 +24527,13 @@
         <v>31550340</v>
       </c>
       <c r="C1114" s="4" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="D1114">
         <v>31550340</v>
       </c>
       <c r="E1114" s="4" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="1115" spans="1:5">
@@ -24531,13 +24544,13 @@
         <v>31550350</v>
       </c>
       <c r="C1115" s="4" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="D1115">
         <v>31550350</v>
       </c>
       <c r="E1115" s="4" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="1116" spans="1:5">
@@ -24548,13 +24561,13 @@
         <v>31550360</v>
       </c>
       <c r="C1116" s="4" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="D1116">
         <v>31550360</v>
       </c>
       <c r="E1116" s="4" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="1117" spans="1:5">
@@ -24565,13 +24578,13 @@
         <v>31550370</v>
       </c>
       <c r="C1117" s="4" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="D1117">
         <v>31550370</v>
       </c>
       <c r="E1117" s="4" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="1118" spans="1:5">
@@ -24582,13 +24595,13 @@
         <v>31550380</v>
       </c>
       <c r="C1118" s="4" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="D1118">
         <v>31550380</v>
       </c>
       <c r="E1118" s="4" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="1119" spans="1:5">
@@ -24599,13 +24612,13 @@
         <v>31570110</v>
       </c>
       <c r="C1119" s="4" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="D1119">
         <v>31570110</v>
       </c>
       <c r="E1119" s="4" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="1120" spans="1:5">
@@ -24616,13 +24629,13 @@
         <v>31570310</v>
       </c>
       <c r="C1120" s="4" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="D1120">
         <v>31570310</v>
       </c>
       <c r="E1120" s="4" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="1121" spans="1:5">
@@ -24633,13 +24646,13 @@
         <v>31570320</v>
       </c>
       <c r="C1121" s="4" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="D1121">
         <v>31570320</v>
       </c>
       <c r="E1121" s="4" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="1122" spans="1:5">
@@ -24650,13 +24663,13 @@
         <v>31570330</v>
       </c>
       <c r="C1122" s="4" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="D1122">
         <v>31570330</v>
       </c>
       <c r="E1122" s="4" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="1123" spans="1:5">
@@ -24667,13 +24680,13 @@
         <v>31570360</v>
       </c>
       <c r="C1123" s="4" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="D1123">
         <v>31570360</v>
       </c>
       <c r="E1123" s="4" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="1124" spans="1:5">
@@ -24684,13 +24697,13 @@
         <v>31570350</v>
       </c>
       <c r="C1124" s="4" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="D1124">
         <v>31570350</v>
       </c>
       <c r="E1124" s="4" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="1125" spans="1:5">
@@ -24701,13 +24714,13 @@
         <v>31580110</v>
       </c>
       <c r="C1125" s="4" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="D1125">
         <v>31580110</v>
       </c>
       <c r="E1125" s="4" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="1126" spans="1:5">
@@ -24718,13 +24731,13 @@
         <v>31580310</v>
       </c>
       <c r="C1126" s="4" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="D1126">
         <v>31580310</v>
       </c>
       <c r="E1126" s="4" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="1127" spans="1:5">
@@ -24735,13 +24748,13 @@
         <v>31580320</v>
       </c>
       <c r="C1127" s="4" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="D1127">
         <v>31580320</v>
       </c>
       <c r="E1127" s="4" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="1128" spans="1:5">
@@ -24752,13 +24765,13 @@
         <v>31580330</v>
       </c>
       <c r="C1128" s="4" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="D1128">
         <v>31580330</v>
       </c>
       <c r="E1128" s="4" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="1129" spans="1:5">
@@ -24769,13 +24782,13 @@
         <v>31580340</v>
       </c>
       <c r="C1129" s="4" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="D1129">
         <v>31580340</v>
       </c>
       <c r="E1129" s="4" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="1130" spans="1:5">
@@ -24786,13 +24799,13 @@
         <v>31580350</v>
       </c>
       <c r="C1130" s="4" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="D1130">
         <v>31580350</v>
       </c>
       <c r="E1130" s="4" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="1131" spans="1:5">
@@ -24803,13 +24816,13 @@
         <v>31580360</v>
       </c>
       <c r="C1131" s="4" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="D1131">
         <v>31580360</v>
       </c>
       <c r="E1131" s="4" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="1132" spans="1:5">
@@ -24820,13 +24833,13 @@
         <v>31580370</v>
       </c>
       <c r="C1132" s="4" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="D1132">
         <v>31580370</v>
       </c>
       <c r="E1132" s="4" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="1133" spans="1:5">
@@ -24837,13 +24850,13 @@
         <v>31580380</v>
       </c>
       <c r="C1133" s="4" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="D1133">
         <v>31580380</v>
       </c>
       <c r="E1133" s="4" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="1134" spans="1:5">
@@ -24854,13 +24867,13 @@
         <v>31580390</v>
       </c>
       <c r="C1134" s="4" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="D1134">
         <v>31580390</v>
       </c>
       <c r="E1134" s="4" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="1135" spans="1:5">
@@ -24871,13 +24884,13 @@
         <v>31580400</v>
       </c>
       <c r="C1135" s="4" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="D1135">
         <v>31580400</v>
       </c>
       <c r="E1135" s="4" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="1136" spans="1:5">
@@ -24888,13 +24901,13 @@
         <v>31580410</v>
       </c>
       <c r="C1136" s="4" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D1136">
         <v>31580410</v>
       </c>
       <c r="E1136" s="4" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="1137" s="5" customFormat="1"/>

</xml_diff>